<commit_message>
skill v0p2 and rtm_gen
</commit_message>
<xml_diff>
--- a/RTM_AI.xlsx
+++ b/RTM_AI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\xingchangchang\ai_evaluation\claude_code\rtm_gen\ai_cc_rtm_gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ADF9A12-C8B6-4F95-B28C-FEBC6736D0DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E576AD1F-3CD9-41EB-A0C4-BDE3EF6267B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR-FL" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="132">
   <si>
     <t>TestPoint分解表格</t>
   </si>
@@ -695,13 +695,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -710,19 +726,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -731,9 +734,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1021,13 +1021,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
@@ -1056,7 +1056,7 @@
       <c r="C3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="30" t="s">
+      <c r="D3" s="15" t="s">
         <v>88</v>
       </c>
       <c r="E3" s="14" t="s">
@@ -1073,7 +1073,7 @@
       <c r="C4" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="15" t="s">
         <v>89</v>
       </c>
       <c r="E4" s="14" t="s">
@@ -1090,7 +1090,7 @@
       <c r="C5" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="15" t="s">
         <v>90</v>
       </c>
       <c r="E5" s="14" t="s">
@@ -1107,7 +1107,7 @@
       <c r="C6" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="15" t="s">
         <v>91</v>
       </c>
       <c r="E6" s="14" t="s">
@@ -1124,7 +1124,7 @@
       <c r="C7" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="15" t="s">
         <v>92</v>
       </c>
       <c r="E7" s="14" t="s">
@@ -1141,7 +1141,7 @@
       <c r="C8" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D8" s="15" t="s">
         <v>93</v>
       </c>
       <c r="E8" s="14" t="s">
@@ -1158,7 +1158,7 @@
       <c r="C9" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="30" t="s">
+      <c r="D9" s="15" t="s">
         <v>94</v>
       </c>
       <c r="E9" s="14" t="s">
@@ -1175,7 +1175,7 @@
       <c r="C10" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="30" t="s">
+      <c r="D10" s="15" t="s">
         <v>95</v>
       </c>
       <c r="E10" s="14" t="s">
@@ -1192,7 +1192,7 @@
       <c r="C11" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="D11" s="30" t="s">
+      <c r="D11" s="15" t="s">
         <v>96</v>
       </c>
       <c r="E11" s="14" t="s">
@@ -1209,7 +1209,7 @@
       <c r="C12" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="30" t="s">
+      <c r="D12" s="15" t="s">
         <v>97</v>
       </c>
       <c r="E12" s="14" t="s">
@@ -1226,7 +1226,7 @@
       <c r="C13" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="D13" s="30" t="s">
+      <c r="D13" s="15" t="s">
         <v>98</v>
       </c>
       <c r="E13" s="14" t="s">
@@ -1243,7 +1243,7 @@
       <c r="C14" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="D14" s="30" t="s">
+      <c r="D14" s="15" t="s">
         <v>99</v>
       </c>
       <c r="E14" s="14" t="s">
@@ -1260,7 +1260,7 @@
       <c r="C15" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="30" t="s">
+      <c r="D15" s="15" t="s">
         <v>100</v>
       </c>
       <c r="E15" s="14" t="s">
@@ -1277,7 +1277,7 @@
       <c r="C16" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="D16" s="30" t="s">
+      <c r="D16" s="15" t="s">
         <v>101</v>
       </c>
       <c r="E16" s="14" t="s">
@@ -1294,7 +1294,7 @@
       <c r="C17" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="D17" s="30" t="s">
+      <c r="D17" s="15" t="s">
         <v>102</v>
       </c>
       <c r="E17" s="14" t="s">
@@ -1311,7 +1311,7 @@
       <c r="C18" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="D18" s="30" t="s">
+      <c r="D18" s="15" t="s">
         <v>103</v>
       </c>
       <c r="E18" s="14" t="s">
@@ -1340,68 +1340,68 @@
       <c r="E21" s="14"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A22" s="26" t="s">
+      <c r="A22" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="23"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
     </row>
     <row r="23" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="B23" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
     </row>
     <row r="24" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="C24" s="23"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="23"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
     </row>
     <row r="25" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
     </row>
     <row r="26" spans="1:5" ht="66.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="C26" s="23"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="23"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
     </row>
     <row r="27" spans="1:5" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="24" t="s">
+      <c r="B27" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A28"/>
@@ -1558,14 +1558,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="17"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="18"/>
     </row>
     <row r="2" spans="1:6" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -1600,8 +1600,12 @@
       <c r="D3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
+      <c r="E3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="4" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A4" s="5" t="s">
@@ -1858,74 +1862,74 @@
       <c r="F19" s="5"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
     </row>
     <row r="24" spans="1:6" ht="54.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="18"/>
     </row>
     <row r="25" spans="1:6" ht="71.099999999999994" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="18"/>
     </row>
     <row r="26" spans="1:6" ht="45.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="18"/>
     </row>
     <row r="27" spans="1:6" ht="38.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="18"/>
     </row>
     <row r="28" spans="1:6" ht="41.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1954,12 +1958,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="17"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -2052,44 +2056,44 @@
       <c r="D12" s="4"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="25" t="s">
         <v>118</v>
       </c>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
     </row>
     <row r="17" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="29" t="s">
         <v>119</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="18"/>
     </row>
     <row r="18" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="30" t="s">
         <v>120</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="18"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A19" s="5"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="17"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="18"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A20" s="5"/>
-      <c r="B20" s="27"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="17"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2117,12 +2121,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="17"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">

</xml_diff>

<commit_message>
skill v0p4(optimized by AI) and rtm
</commit_message>
<xml_diff>
--- a/RTM_AI.xlsx
+++ b/RTM_AI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\xingchangchang\ai_evaluation\claude_code\rtm_gen\ai_cc_rtm_gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E576AD1F-3CD9-41EB-A0C4-BDE3EF6267B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A14264B-4C55-4C2B-8749-2CA9F70D6B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="131">
   <si>
     <t>TestPoint分解表格</t>
   </si>
@@ -277,9 +277,6 @@
   </si>
   <si>
     <t>xxx</t>
-  </si>
-  <si>
-    <t>TP_017</t>
   </si>
   <si>
     <t>填写说明</t>
@@ -416,25 +413,6 @@
   <si>
     <t xml:space="preserve">1.检查频率值是否正确：连续采集时钟上升沿和下降沿并计算实际频率/周期，判断是否处于目标频率的允许误差范围内（±1%）；
 2.检查时钟稳定性：通过连续采样周期，对比相邻两个周期的频率偏差是否在3%内。
-</t>
-  </si>
-  <si>
-    <t>status_reg_check</t>
-  </si>
-  <si>
-    <t xml:space="preserve">在IP解复位后的每个cycle，对IP内部状态寄存器和建模得到的状态进行check：
-1、通道使能寄存器chenreg
-2、通道任务完成原始中断状态寄存器rawtfr_ch
-3、通道任务传输异常原始中断状态寄存器rawerr_ch
-4、通道安全访问异常原始中断状态寄存器rawnsec_ch
-5、
-通道访问异常中断状态寄存器rawacc_ch
-6、公共寄存器组的安全访问异常原始中断寄存器rawcnnsec
-7、公共寄存器组的访问异常原始中断寄存器rawcmacc
-8、通道任务完成mask后的中断状态寄存器statustfr
-9、通道任务传输异常mask后的中断状态寄存器statuserr
-10、通道安全访问异常mask后的中断状态寄存器statusnsec
-11、公共寄存器组的安全访问异常mask后的中断状态寄存器statuscmnsec
 </t>
   </si>
   <si>
@@ -510,12 +488,33 @@
   <si>
     <t>TC_004</t>
   </si>
+  <si>
+    <t xml:space="preserve">在IP解复位后的每个cycle，对IP内部状态寄存器和建模得到的状态进行check：
+1、通道使能寄存器chenreg
+2、通道任务完成原始中断状态寄存器rawtfr_ch
+3、通道任务传输异常原始中断状态寄存器rawerr_ch
+4、通道安全访问异常原始中断状态寄存器rawnsec_ch
+5、
+通道访问异常中断状态寄存器rawacc_ch
+6、公共寄存器组的安全访问异常原始中断寄存器rawcnnsec
+7、公共寄存器组的访问异常原始中断寄存器rawcmacc
+8、通道任务完成mask后的中断状态寄存器statustfr
+9、通道任务传输异常mask后的中断状态寄存器statuserr
+10、通道安全访问异常mask后的中断状态寄存器statusnsec
+11、公共寄存器组的安全访问异常mask后的中断状态寄存器statuscmnsec
+</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>status_reg_check</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -548,6 +547,22 @@
     <font>
       <sz val="9"/>
       <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -653,7 +668,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -698,11 +713,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -715,16 +749,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1021,26 +1045,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A1" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
+      <c r="A1" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="D2" s="10" t="s">
         <v>85</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>86</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>3</v>
@@ -1048,7 +1072,7 @@
     </row>
     <row r="3" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A3" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>8</v>
@@ -1057,7 +1081,7 @@
         <v>7</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>9</v>
@@ -1065,7 +1089,7 @@
     </row>
     <row r="4" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A4" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>13</v>
@@ -1074,7 +1098,7 @@
         <v>12</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>14</v>
@@ -1082,7 +1106,7 @@
     </row>
     <row r="5" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A5" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>18</v>
@@ -1091,7 +1115,7 @@
         <v>17</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>19</v>
@@ -1099,7 +1123,7 @@
     </row>
     <row r="6" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A6" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>23</v>
@@ -1108,7 +1132,7 @@
         <v>22</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>24</v>
@@ -1116,7 +1140,7 @@
     </row>
     <row r="7" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A7" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>23</v>
@@ -1125,7 +1149,7 @@
         <v>27</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>28</v>
@@ -1133,7 +1157,7 @@
     </row>
     <row r="8" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A8" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>31</v>
@@ -1142,7 +1166,7 @@
         <v>30</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>32</v>
@@ -1150,7 +1174,7 @@
     </row>
     <row r="9" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A9" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>31</v>
@@ -1159,7 +1183,7 @@
         <v>34</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>35</v>
@@ -1167,7 +1191,7 @@
     </row>
     <row r="10" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A10" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>38</v>
@@ -1176,7 +1200,7 @@
         <v>37</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E10" s="14" t="s">
         <v>39</v>
@@ -1184,7 +1208,7 @@
     </row>
     <row r="11" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A11" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>42</v>
@@ -1193,7 +1217,7 @@
         <v>41</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E11" s="14" t="s">
         <v>43</v>
@@ -1201,7 +1225,7 @@
     </row>
     <row r="12" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A12" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>46</v>
@@ -1210,7 +1234,7 @@
         <v>45</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E12" s="14" t="s">
         <v>47</v>
@@ -1218,7 +1242,7 @@
     </row>
     <row r="13" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A13" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>50</v>
@@ -1227,7 +1251,7 @@
         <v>49</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E13" s="14" t="s">
         <v>51</v>
@@ -1235,7 +1259,7 @@
     </row>
     <row r="14" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A14" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B14" s="12" t="s">
         <v>54</v>
@@ -1244,7 +1268,7 @@
         <v>53</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E14" s="14" t="s">
         <v>55</v>
@@ -1252,7 +1276,7 @@
     </row>
     <row r="15" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A15" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>58</v>
@@ -1261,7 +1285,7 @@
         <v>57</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E15" s="14" t="s">
         <v>59</v>
@@ -1269,7 +1293,7 @@
     </row>
     <row r="16" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A16" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>62</v>
@@ -1278,7 +1302,7 @@
         <v>61</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E16" s="14" t="s">
         <v>63</v>
@@ -1286,7 +1310,7 @@
     </row>
     <row r="17" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A17" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>66</v>
@@ -1295,7 +1319,7 @@
         <v>65</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>67</v>
@@ -1303,7 +1327,7 @@
     </row>
     <row r="18" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A18" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>70</v>
@@ -1312,7 +1336,7 @@
         <v>69</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E18" s="14" t="s">
         <v>71</v>
@@ -1340,68 +1364,68 @@
       <c r="E21" s="14"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A22" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
+      <c r="A22" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
     </row>
     <row r="23" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="B23" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
+        <v>82</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
     </row>
     <row r="24" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="B24" s="19" t="s">
-        <v>105</v>
-      </c>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
+        <v>83</v>
+      </c>
+      <c r="B24" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
     </row>
     <row r="25" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="B25" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
+        <v>84</v>
+      </c>
+      <c r="B25" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
     </row>
     <row r="26" spans="1:5" ht="66.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="B26" s="19" t="s">
-        <v>107</v>
-      </c>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
+        <v>85</v>
+      </c>
+      <c r="B26" s="26" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
     </row>
     <row r="27" spans="1:5" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
+      <c r="B27" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A28"/>
@@ -1558,14 +1582,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:6" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -1604,7 +1628,7 @@
         <v>11</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="54" x14ac:dyDescent="0.15">
@@ -1848,88 +1872,82 @@
       <c r="F18" s="5"/>
     </row>
     <row r="19" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>74</v>
-      </c>
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
       <c r="D19" s="4"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A23" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
+      <c r="A23" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
     </row>
     <row r="24" spans="1:6" ht="54.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B24" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="18"/>
+      <c r="B24" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="21"/>
     </row>
     <row r="25" spans="1:6" ht="71.099999999999994" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B25" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="18"/>
+      <c r="B25" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="21"/>
     </row>
     <row r="26" spans="1:6" ht="45.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B26" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="18"/>
+      <c r="B26" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="21"/>
     </row>
     <row r="27" spans="1:6" ht="38.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="18"/>
+      <c r="B27" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="21"/>
     </row>
     <row r="28" spans="1:6" ht="41.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="B28" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="18"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1948,7 +1966,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18.875" style="9" customWidth="1"/>
@@ -1958,25 +1976,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="18"/>
+      <c r="A1" s="22" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="60.95" customHeight="1" x14ac:dyDescent="0.15">
@@ -1984,10 +2002,10 @@
         <v>11</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>114</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>115</v>
       </c>
       <c r="D3" s="4"/>
     </row>
@@ -1995,11 +2013,11 @@
       <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>117</v>
+      <c r="B4" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>129</v>
       </c>
       <c r="D4" s="4"/>
     </row>
@@ -2008,7 +2026,7 @@
         <v>21</v>
       </c>
       <c r="B5" s="5"/>
-      <c r="C5" s="4"/>
+      <c r="C5" s="6"/>
       <c r="D5" s="4"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.15">
@@ -2016,93 +2034,165 @@
         <v>26</v>
       </c>
       <c r="B6" s="5"/>
-      <c r="C6" s="4"/>
+      <c r="C6" s="6"/>
       <c r="D6" s="4"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="A7" s="12"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="A8" s="12"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="A9" s="12"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="14"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
+      <c r="A10" s="12"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="14"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="A11" s="12"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+      <c r="A12" s="12"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="14"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="14"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A14" s="12"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="14"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="14"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A16" s="25" t="s">
-        <v>118</v>
-      </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-    </row>
-    <row r="17" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="B17" s="29" t="s">
-        <v>119</v>
-      </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="18"/>
-    </row>
-    <row r="18" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="B18" s="30" t="s">
-        <v>120</v>
-      </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="18"/>
+      <c r="A16" s="12"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="14"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="14"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="14"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A19" s="5"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="18"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="4"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A20" s="5"/>
-      <c r="B20" s="28"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="18"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="4"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="4"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="4"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A28" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="B28" s="24"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+    </row>
+    <row r="29" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A29" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B29" s="32" t="s">
+        <v>116</v>
+      </c>
+      <c r="C29" s="20"/>
+      <c r="D29" s="21"/>
+    </row>
+    <row r="30" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A30" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B30" s="33" t="s">
+        <v>117</v>
+      </c>
+      <c r="C30" s="20"/>
+      <c r="D30" s="21"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A31" s="5"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="21"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A32" s="5"/>
+      <c r="B32" s="31"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B32:D32"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="A28:D28"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2111,7 +2201,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="13.75" style="9" customWidth="1"/>
@@ -2121,108 +2211,180 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="16" t="s">
-        <v>121</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="18"/>
+      <c r="A1" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="98.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:4" ht="192" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D4" s="4"/>
     </row>
     <row r="5" spans="1:4" ht="54.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>73</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="4"/>
+      <c r="C6" s="3"/>
       <c r="D6" s="4"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+    <row r="7" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="14"/>
+    </row>
+    <row r="8" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="14"/>
+    </row>
+    <row r="9" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="14"/>
+    </row>
+    <row r="10" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="14"/>
+    </row>
+    <row r="11" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="14"/>
+    </row>
+    <row r="12" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="14"/>
+    </row>
+    <row r="13" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A13" s="16"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="14"/>
+    </row>
+    <row r="14" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="14"/>
+    </row>
+    <row r="15" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="14"/>
+    </row>
+    <row r="16" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="16"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="14"/>
+    </row>
+    <row r="17" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="16"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="14"/>
+    </row>
+    <row r="18" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A18" s="16"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="14"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="4"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="4"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="4"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
skill v0p5(optimized by AI) and rtm(gen in plan mode)
</commit_message>
<xml_diff>
--- a/RTM_AI.xlsx
+++ b/RTM_AI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\xingchangchang\ai_evaluation\claude_code\rtm_gen\ai_cc_rtm_gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A14264B-4C55-4C2B-8749-2CA9F70D6B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172150DD-F50A-42EC-87F9-8C20B0AAD424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="115">
   <si>
     <t>TestPoint分解表格</t>
   </si>
@@ -53,14 +53,6 @@
   </si>
   <si>
     <t>TP_001</t>
-  </si>
-  <si>
-    <t>条件：配置clk_i时钟频率为100MHz，验证模块时钟域同步性。
-激励：连续发送AHB_RD32和AHB_WR32命令，覆盖1-bit和4-bit两种lane模式。
-期望：所有命令在100MHz频率下正确执行，协议采样、状态机控制和AHB-Lite主接口同域工作正常，无时序违例。</t>
-  </si>
-  <si>
-    <t>CHK_001</t>
   </si>
   <si>
     <t>FL_002_001</t>
@@ -77,9 +69,6 @@
 期望：复位后状态机处于IDLE，CTRL寄存器默认值正确，STATUS/LAST_ERR清零，无残留状态。</t>
   </si>
   <si>
-    <t>CHK_002</t>
-  </si>
-  <si>
     <t>FL_003_001</t>
   </si>
   <si>
@@ -94,9 +83,6 @@
 期望：CSR读写正确，VERSION返回预期值，CTRL配置生效，STATUS/LAST_ERR反映正确状态。</t>
   </si>
   <si>
-    <t>CHK_003</t>
-  </si>
-  <si>
     <t>FL_004_001</t>
   </si>
   <si>
@@ -111,9 +97,6 @@
 期望：模块正确执行功能命令，协议采用半双工模式，CSR访问与AHB-Lite单次读写正常。</t>
   </si>
   <si>
-    <t>CHK_004</t>
-  </si>
-  <si>
     <t>FL_004_002</t>
   </si>
   <si>
@@ -274,9 +257,6 @@
     <t>条件：模块使能，AHB总线空闲。
 激励：1) 发送AHB_WR32命令，验证haddr_o/hwrite_o/htrans_o/hsize_o/hburst_o/hwdata_o输出正确；2) 发送AHB_RD32命令，验证hrdata_i/hready_i/hresp_i输入正确处理；3) 验证htrans_o仅输出IDLE/NONSEQ；4) 验证hsize_o固定为WORD(32-bit)；5) 验证hburst_o固定为SINGLE。
 期望：AHB-Lite Master接口符合规范，单次读写事务正确，信号时序满足AHB协议要求。</t>
-  </si>
-  <si>
-    <t>xxx</t>
   </si>
   <si>
     <t>填写说明</t>
@@ -408,14 +388,6 @@
     <t>备注</t>
   </si>
   <si>
-    <t>clk_freq_check</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.检查频率值是否正确：连续采集时钟上升沿和下降沿并计算实际频率/周期，判断是否处于目标频率的允许误差范围内（±1%）；
-2.检查时钟稳定性：通过连续采样周期，对比相邻两个周期的频率偏差是否在3%内。
-</t>
-  </si>
-  <si>
     <t>填写要求</t>
   </si>
   <si>
@@ -439,74 +411,9 @@
     <t>TC 描述</t>
   </si>
   <si>
-    <t>TC_001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">配置条件：
-//对配置寄存器或接口控制信号进行描述
-输入激励：
-1/对接口激励进行描述
-期望结果：
-// 描述逻辑处理期望的结果，以及check点
-coverage check点：
-//如果通过随机测试，功能模型建模来确认对测试点的覆盖，需要描述功能模型的功能。如果通过直接用例来覆盖测试点，则不需要收集功
-能覆盖率，该部分内容不用描述。
-</t>
-  </si>
-  <si>
-    <t>TC_002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">配置条件：
-1.RSIO模块解复位初始化接收通路；
-仅配置lane0，其它lane无效：1）解复位并使能接受通道lane0，并配置lane0数据通路正确接收数据；2）复位并不使能lane0通路；3)
-再解复位使能lane0，并配置lane0数据通路正确接收数据；
-3.仅配置lane1，其它lane无效：配置过程同上lane0
-4.仅配置lane2，其它lane无效：配置过程同上lane0
-5.仅配置lane3，其它lane无效：配置过程同上lane0
-其它：以上测试过程中，不关心的配置或接口控制信号随机
-输入激励：
-2.对应lane0通路，依次按照使能的情况，发送方依次输入激励数据包和参考时钟；
-3.对应lane1通路，依次按照使能的情况，发送方依次输入激励数据包和参考时钟；
-4.对应lane2通路，依次按照使能的情况，发送方依次输入激励数据包和参考时钟；
-5.对应lane3通路，依次按照使能的情况，发送方依次输入激励数据包和参考时钟；
-期望结果：
-2.lane0使能期间，能正确接受到发送方发来的数据，不使能期间无数据；其它lane同道无数据；
-3.lane1使能期间，能正确接受到发送方发来的数据，不使能期间无数据；其它lane同道无数据；
-4.lane2使能期间，能正确接受到发送方发来的数据，不使能期间无数据；其它lane同道无数据；
-5.lane3使能期间，能正确接受到发送方发来的数据，不使能期间无数据；其它lane同道无数据；
-coverage check点：
-直接用例覆盖，不收功能覆盖率
-</t>
-  </si>
-  <si>
-    <t>TC_003</t>
-  </si>
-  <si>
-    <t>同一类别的多个TC（如遍历不同分辨率）需逐个列出，不能合并为一个TC。但不必逐项详述，以一个典型TC作为基准进行完整定义，其余TC仅描述与基准TC的差异（相同部分可以写“其他配置和激励同TC_xxx”）。</t>
-  </si>
-  <si>
-    <t>TC_004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">在IP解复位后的每个cycle，对IP内部状态寄存器和建模得到的状态进行check：
-1、通道使能寄存器chenreg
-2、通道任务完成原始中断状态寄存器rawtfr_ch
-3、通道任务传输异常原始中断状态寄存器rawerr_ch
-4、通道安全访问异常原始中断状态寄存器rawnsec_ch
-5、
-通道访问异常中断状态寄存器rawacc_ch
-6、公共寄存器组的安全访问异常原始中断寄存器rawcnnsec
-7、公共寄存器组的访问异常原始中断寄存器rawcmacc
-8、通道任务完成mask后的中断状态寄存器statustfr
-9、通道任务传输异常mask后的中断状态寄存器statuserr
-10、通道安全访问异常mask后的中断状态寄存器statusnsec
-11、公共寄存器组的安全访问异常mask后的中断状态寄存器statuscmnsec
-</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>status_reg_check</t>
+    <t>条件：配置clk_i时钟频率为100MHz，验证模块时钟域同步性。
+激励：连续发送AHB_RD32和AHB_WR32命令，覆盖1-bit和4-bit两种lane模式。
+期望：所有命令在100MHz频率下正确执行，协议采样、状态机控制和AHB-Lite主接口同域工作正常。</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -668,7 +575,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -758,6 +665,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1046,7 +956,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A1" s="29" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -1055,16 +965,16 @@
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>3</v>
@@ -1072,7 +982,7 @@
     </row>
     <row r="3" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A3" s="12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>8</v>
@@ -1081,7 +991,7 @@
         <v>7</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>9</v>
@@ -1089,257 +999,257 @@
     </row>
     <row r="4" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A4" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C4" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="E4" s="14" t="s">
         <v>12</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A5" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A6" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A7" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B7" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="E7" s="14" t="s">
         <v>23</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A8" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>92</v>
-      </c>
       <c r="E8" s="14" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A9" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A10" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A11" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A12" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A13" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A14" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A15" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A16" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="27" x14ac:dyDescent="0.15">
       <c r="A17" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A18" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.15">
@@ -1365,7 +1275,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A22" s="30" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="27"/>
@@ -1374,10 +1284,10 @@
     </row>
     <row r="23" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="12" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B23" s="28" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C23" s="27"/>
       <c r="D23" s="27"/>
@@ -1385,10 +1295,10 @@
     </row>
     <row r="24" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="12" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C24" s="27"/>
       <c r="D24" s="27"/>
@@ -1396,10 +1306,10 @@
     </row>
     <row r="25" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="12" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C25" s="27"/>
       <c r="D25" s="27"/>
@@ -1407,10 +1317,10 @@
     </row>
     <row r="26" spans="1:5" ht="66.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="12" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C26" s="27"/>
       <c r="D26" s="27"/>
@@ -1421,7 +1331,7 @@
         <v>3</v>
       </c>
       <c r="B27" s="28" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C27" s="27"/>
       <c r="D27" s="27"/>
@@ -1621,252 +1531,248 @@
       <c r="C3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>122</v>
-      </c>
+      <c r="D3" s="34" t="s">
+        <v>114</v>
+      </c>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
     </row>
     <row r="4" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="D4" s="7" t="s">
         <v>13</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>15</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
     </row>
     <row r="5" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>17</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>20</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
     </row>
     <row r="6" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A6" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
     </row>
     <row r="7" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A7" s="5" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>28</v>
-      </c>
       <c r="D7" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
     </row>
     <row r="8" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A8" s="5" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
     </row>
     <row r="9" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A9" s="5" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>31</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>36</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
     </row>
     <row r="10" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A10" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
     </row>
     <row r="11" spans="1:6" ht="67.5" x14ac:dyDescent="0.15">
       <c r="A11" s="5" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
     </row>
     <row r="12" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A12" s="5" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
     </row>
     <row r="13" spans="1:6" ht="81" x14ac:dyDescent="0.15">
       <c r="A13" s="5" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
     </row>
     <row r="14" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A14" s="5" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
     </row>
     <row r="15" spans="1:6" ht="67.5" x14ac:dyDescent="0.15">
       <c r="A15" s="5" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
     </row>
     <row r="16" spans="1:6" ht="54" x14ac:dyDescent="0.15">
       <c r="A16" s="5" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
     </row>
     <row r="17" spans="1:6" ht="67.5" x14ac:dyDescent="0.15">
       <c r="A17" s="5" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
     </row>
     <row r="18" spans="1:6" ht="67.5" x14ac:dyDescent="0.15">
       <c r="A18" s="5" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
@@ -1881,7 +1787,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A23" s="23" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B23" s="24"/>
       <c r="C23" s="24"/>
@@ -1894,7 +1800,7 @@
         <v>1</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C24" s="20"/>
       <c r="D24" s="20"/>
@@ -1906,7 +1812,7 @@
         <v>2</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C25" s="20"/>
       <c r="D25" s="20"/>
@@ -1918,7 +1824,7 @@
         <v>3</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C26" s="20"/>
       <c r="D26" s="20"/>
@@ -1930,7 +1836,7 @@
         <v>6</v>
       </c>
       <c r="B27" s="25" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C27" s="20"/>
       <c r="D27" s="20"/>
@@ -1939,10 +1845,10 @@
     </row>
     <row r="28" spans="1:6" ht="41.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="5" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B28" s="25" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C28" s="20"/>
       <c r="D28" s="20"/>
@@ -1977,7 +1883,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A1" s="22" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -1985,54 +1891,38 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="60.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>114</v>
-      </c>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="6"/>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" spans="1:4" ht="155.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>130</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>129</v>
-      </c>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A4" s="5"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="17"/>
       <c r="D4" s="4"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A5" s="5" t="s">
-        <v>21</v>
-      </c>
+      <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="6"/>
       <c r="D5" s="4"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A6" s="5" t="s">
-        <v>26</v>
-      </c>
+      <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="6"/>
       <c r="D6" s="4"/>
@@ -2147,7 +2037,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A28" s="23" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="B28" s="24"/>
       <c r="C28" s="24"/>
@@ -2155,20 +2045,20 @@
     </row>
     <row r="29" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="5" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B29" s="32" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="C29" s="20"/>
       <c r="D29" s="21"/>
     </row>
     <row r="30" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="5" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C30" s="20"/>
       <c r="D30" s="21"/>
@@ -2212,7 +2102,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A1" s="22" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -2220,131 +2110,109 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="98.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>123</v>
-      </c>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="3"/>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" spans="1:4" ht="192" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>125</v>
-      </c>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="3"/>
       <c r="D4" s="4"/>
     </row>
-    <row r="5" spans="1:4" ht="54.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>127</v>
-      </c>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="3"/>
       <c r="D5" s="4"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A6" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>73</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
       <c r="C6" s="3"/>
       <c r="D6" s="4"/>
     </row>
-    <row r="7" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A7" s="16"/>
       <c r="B7" s="16"/>
       <c r="C7" s="3"/>
       <c r="D7" s="14"/>
     </row>
-    <row r="8" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
       <c r="C8" s="3"/>
       <c r="D8" s="14"/>
     </row>
-    <row r="9" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A9" s="16"/>
       <c r="B9" s="16"/>
       <c r="C9" s="3"/>
       <c r="D9" s="14"/>
     </row>
-    <row r="10" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A10" s="16"/>
       <c r="B10" s="16"/>
       <c r="C10" s="3"/>
       <c r="D10" s="14"/>
     </row>
-    <row r="11" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A11" s="16"/>
       <c r="B11" s="16"/>
       <c r="C11" s="3"/>
       <c r="D11" s="14"/>
     </row>
-    <row r="12" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A12" s="16"/>
       <c r="B12" s="16"/>
       <c r="C12" s="3"/>
       <c r="D12" s="14"/>
     </row>
-    <row r="13" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A13" s="16"/>
       <c r="B13" s="16"/>
       <c r="C13" s="3"/>
       <c r="D13" s="14"/>
     </row>
-    <row r="14" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A14" s="16"/>
       <c r="B14" s="16"/>
       <c r="C14" s="3"/>
       <c r="D14" s="14"/>
     </row>
-    <row r="15" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A15" s="16"/>
       <c r="B15" s="16"/>
       <c r="C15" s="3"/>
       <c r="D15" s="14"/>
     </row>
-    <row r="16" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A16" s="16"/>
       <c r="B16" s="16"/>
       <c r="C16" s="3"/>
       <c r="D16" s="14"/>
     </row>
-    <row r="17" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A17" s="16"/>
       <c r="B17" s="16"/>
       <c r="C17" s="3"/>
       <c r="D17" s="14"/>
     </row>
-    <row r="18" spans="1:4" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A18" s="16"/>
       <c r="B18" s="16"/>
       <c r="C18" s="3"/>

</xml_diff>

<commit_message>
skill v0p9(add ref) and rtm(plan mode)
</commit_message>
<xml_diff>
--- a/RTM_AI.xlsx
+++ b/RTM_AI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\xingchangchang\ai_evaluation\claude_code\rtm_gen\ai_cc_rtm_gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172150DD-F50A-42EC-87F9-8C20B0AAD424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCF3F90-E61B-4167-B968-4EF09B902314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR-FL" sheetId="1" r:id="rId1"/>
@@ -433,6 +433,7 @@
       <sz val="8"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -440,6 +441,7 @@
       <sz val="6"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -448,12 +450,14 @@
       <sz val="11"/>
       <color theme="0"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -575,7 +579,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -628,6 +632,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -666,7 +673,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -955,13 +965,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
@@ -1274,68 +1284,68 @@
       <c r="E21" s="14"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A22" s="30" t="s">
+      <c r="A22" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="B22" s="27"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
     </row>
     <row r="23" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="29" t="s">
         <v>97</v>
       </c>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
     </row>
     <row r="24" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="B24" s="26" t="s">
+      <c r="B24" s="27" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
     </row>
     <row r="25" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B25" s="28" t="s">
+      <c r="B25" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="28"/>
     </row>
     <row r="26" spans="1:5" ht="66.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="B26" s="26" t="s">
+      <c r="B26" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="28"/>
     </row>
     <row r="27" spans="1:5" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="28" t="s">
+      <c r="B27" s="29" t="s">
         <v>101</v>
       </c>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="28"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A28"/>
@@ -1492,14 +1502,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="21"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="22"/>
     </row>
     <row r="2" spans="1:6" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -1531,7 +1541,7 @@
       <c r="C3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="D3" s="19" t="s">
         <v>114</v>
       </c>
       <c r="E3" s="5"/>
@@ -1786,74 +1796,74 @@
       <c r="F19" s="5"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A23" s="23" t="s">
+      <c r="A23" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
     </row>
     <row r="24" spans="1:6" ht="54.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="22"/>
     </row>
     <row r="25" spans="1:6" ht="71.099999999999994" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="21"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="22"/>
     </row>
     <row r="26" spans="1:6" ht="45.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="B26" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="22"/>
     </row>
     <row r="27" spans="1:6" ht="38.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="25" t="s">
+      <c r="B27" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="22"/>
     </row>
     <row r="28" spans="1:6" ht="41.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B28" s="25" t="s">
+      <c r="B28" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1872,7 +1882,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18.875" style="9" customWidth="1"/>
@@ -1882,12 +1892,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="21"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="22"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -1990,99 +2000,147 @@
     <row r="17" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A17" s="12"/>
       <c r="B17" s="12"/>
-      <c r="C17" s="6"/>
+      <c r="C17" s="36"/>
       <c r="D17" s="14"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A18" s="12"/>
       <c r="B18" s="12"/>
-      <c r="C18" s="6"/>
+      <c r="C18" s="36"/>
       <c r="D18" s="14"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="4"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="14"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="4"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="14"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="4"/>
+      <c r="A21" s="12"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="14"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="4"/>
+      <c r="A22" s="12"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="14"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="4"/>
+      <c r="A23" s="12"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="14"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="4"/>
+      <c r="A24" s="12"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="14"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A25" s="12"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="14"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A26" s="12"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="14"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A27" s="5"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="4"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A28" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-    </row>
-    <row r="29" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B29" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="C29" s="20"/>
-      <c r="D29" s="21"/>
-    </row>
-    <row r="30" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B30" s="33" t="s">
-        <v>109</v>
-      </c>
-      <c r="C30" s="20"/>
-      <c r="D30" s="21"/>
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="4"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="4"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A30" s="5"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="4"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A31" s="5"/>
-      <c r="B31" s="31"/>
-      <c r="C31" s="20"/>
-      <c r="D31" s="21"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="4"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A32" s="5"/>
-      <c r="B32" s="31"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="21"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="4"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A36" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="B36" s="25"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+    </row>
+    <row r="37" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A37" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B37" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="C37" s="21"/>
+      <c r="D37" s="22"/>
+    </row>
+    <row r="38" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A38" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B38" s="34" t="s">
+        <v>109</v>
+      </c>
+      <c r="C38" s="21"/>
+      <c r="D38" s="22"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A39" s="5"/>
+      <c r="B39" s="32"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="22"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A40" s="5"/>
+      <c r="B40" s="32"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B40:D40"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="A36:D36"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2091,7 +2149,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="13.75" style="9" customWidth="1"/>
@@ -2101,12 +2159,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="21"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="22"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -2149,110 +2207,218 @@
     <row r="7" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A7" s="16"/>
       <c r="B7" s="16"/>
-      <c r="C7" s="3"/>
+      <c r="C7" s="35"/>
       <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
-      <c r="C8" s="3"/>
+      <c r="C8" s="35"/>
       <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A9" s="16"/>
       <c r="B9" s="16"/>
-      <c r="C9" s="3"/>
+      <c r="C9" s="35"/>
       <c r="D9" s="14"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A10" s="16"/>
       <c r="B10" s="16"/>
-      <c r="C10" s="3"/>
+      <c r="C10" s="35"/>
       <c r="D10" s="14"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A11" s="16"/>
       <c r="B11" s="16"/>
-      <c r="C11" s="3"/>
+      <c r="C11" s="35"/>
       <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A12" s="16"/>
       <c r="B12" s="16"/>
-      <c r="C12" s="3"/>
+      <c r="C12" s="35"/>
       <c r="D12" s="14"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A13" s="16"/>
       <c r="B13" s="16"/>
-      <c r="C13" s="3"/>
+      <c r="C13" s="35"/>
       <c r="D13" s="14"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A14" s="16"/>
       <c r="B14" s="16"/>
-      <c r="C14" s="3"/>
+      <c r="C14" s="35"/>
       <c r="D14" s="14"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A15" s="16"/>
       <c r="B15" s="16"/>
-      <c r="C15" s="3"/>
+      <c r="C15" s="35"/>
       <c r="D15" s="14"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A16" s="16"/>
       <c r="B16" s="16"/>
-      <c r="C16" s="3"/>
+      <c r="C16" s="35"/>
       <c r="D16" s="14"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A17" s="16"/>
       <c r="B17" s="16"/>
-      <c r="C17" s="3"/>
+      <c r="C17" s="35"/>
       <c r="D17" s="14"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A18" s="16"/>
       <c r="B18" s="16"/>
-      <c r="C18" s="3"/>
+      <c r="C18" s="35"/>
       <c r="D18" s="14"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="4"/>
+      <c r="A19" s="16"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="14"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="4"/>
+      <c r="A20" s="16"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="14"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="4"/>
+      <c r="A21" s="16"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="14"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="4"/>
+      <c r="A22" s="16"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="14"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="4"/>
+      <c r="A23" s="16"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="14"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="4"/>
+      <c r="A24" s="16"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="14"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A25" s="16"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="14"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A26" s="16"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="14"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A27" s="16"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="14"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A28" s="16"/>
+      <c r="B28" s="16"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="14"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A29" s="16"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="14"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A30" s="16"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="14"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A31" s="16"/>
+      <c r="B31" s="16"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="14"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A32" s="16"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="14"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A33" s="16"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="14"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A34" s="16"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="14"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A35" s="16"/>
+      <c r="B35" s="16"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="14"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A36" s="16"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="14"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A37" s="4"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="4"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A38" s="4"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="4"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="4"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="4"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="4"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A42" s="4"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
skill v1p0(follow template modify) and rtm(plan mode)
</commit_message>
<xml_diff>
--- a/RTM_AI.xlsx
+++ b/RTM_AI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\xingchangchang\ai_evaluation\claude_code\rtm_gen\ai_cc_rtm_gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCF3F90-E61B-4167-B968-4EF09B902314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C1AD95-4498-4F97-93C7-3B9C6DCB0C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DR-FL" sheetId="1" r:id="rId1"/>
@@ -579,7 +579,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -636,21 +636,27 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -665,19 +671,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -965,13 +962,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
@@ -1284,68 +1281,68 @@
       <c r="E21" s="14"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A22" s="31" t="s">
+      <c r="A22" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
     </row>
     <row r="23" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="29" t="s">
+      <c r="B23" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
     </row>
     <row r="24" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="B24" s="27" t="s">
+      <c r="B24" s="29" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="28"/>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
     </row>
     <row r="25" spans="1:5" ht="42.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B25" s="29" t="s">
+      <c r="B25" s="31" t="s">
         <v>99</v>
       </c>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
     </row>
     <row r="26" spans="1:5" ht="66.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="B26" s="27" t="s">
+      <c r="B26" s="29" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
+      <c r="C26" s="30"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="30"/>
     </row>
     <row r="27" spans="1:5" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="29" t="s">
+      <c r="B27" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
+      <c r="C27" s="30"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A28"/>
@@ -1502,14 +1499,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="23"/>
     </row>
     <row r="2" spans="1:6" ht="29.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -1796,74 +1793,74 @@
       <c r="F19" s="5"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="A23" s="24" t="s">
+      <c r="A23" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
     </row>
     <row r="24" spans="1:6" ht="54.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="23"/>
     </row>
     <row r="25" spans="1:6" ht="71.099999999999994" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="23"/>
     </row>
     <row r="26" spans="1:6" ht="45.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="23"/>
     </row>
     <row r="27" spans="1:6" ht="38.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="B27" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="23"/>
     </row>
     <row r="28" spans="1:6" ht="41.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" s="35" t="s">
         <v>74</v>
       </c>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1882,7 +1879,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18.875" style="9" customWidth="1"/>
@@ -1892,12 +1889,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="22"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="23"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -1931,216 +1928,54 @@
       <c r="C5" s="6"/>
       <c r="D5" s="4"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="14"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="14"/>
-    </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="14"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="14"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="14"/>
+      <c r="A9" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+    </row>
+    <row r="10" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" s="22"/>
+      <c r="D10" s="23"/>
+    </row>
+    <row r="11" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="C11" s="22"/>
+      <c r="D11" s="23"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="14"/>
+      <c r="A12" s="5"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="23"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="14"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="14"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="14"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="14"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="14"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="14"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="14"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="14"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="14"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A22" s="12"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="14"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="36"/>
-      <c r="D23" s="14"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="36"/>
-      <c r="D24" s="14"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="14"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A26" s="12"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="14"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A27" s="5"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="4"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="4"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="4"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="4"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="4"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A32" s="5"/>
-      <c r="B32" s="5"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="4"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A36" s="24" t="s">
-        <v>107</v>
-      </c>
-      <c r="B36" s="25"/>
-      <c r="C36" s="25"/>
-      <c r="D36" s="25"/>
-    </row>
-    <row r="37" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A37" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B37" s="33" t="s">
-        <v>108</v>
-      </c>
-      <c r="C37" s="21"/>
-      <c r="D37" s="22"/>
-    </row>
-    <row r="38" spans="1:4" ht="69.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A38" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B38" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="C38" s="21"/>
-      <c r="D38" s="22"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A39" s="5"/>
-      <c r="B39" s="32"/>
-      <c r="C39" s="21"/>
-      <c r="D39" s="22"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A40" s="5"/>
-      <c r="B40" s="32"/>
-      <c r="C40" s="21"/>
-      <c r="D40" s="22"/>
+      <c r="A13" s="5"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B13:D13"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="A9:D9"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2149,7 +1984,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="13.75" style="9" customWidth="1"/>
@@ -2159,12 +1994,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="22"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="23"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
@@ -2207,218 +2042,8 @@
     <row r="7" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A7" s="16"/>
       <c r="B7" s="16"/>
-      <c r="C7" s="35"/>
+      <c r="C7" s="20"/>
       <c r="D7" s="14"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A8" s="16"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="14"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A9" s="16"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="14"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A10" s="16"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="14"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A11" s="16"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="14"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A12" s="16"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="14"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A13" s="16"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="14"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A14" s="16"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="14"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A15" s="16"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="14"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A16" s="16"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="14"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A17" s="16"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="14"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A18" s="16"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="14"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A19" s="16"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="14"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A20" s="16"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="14"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A21" s="16"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="14"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A22" s="16"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="14"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A23" s="16"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="14"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A24" s="16"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="14"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A25" s="16"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="14"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A26" s="16"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="14"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="14"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A28" s="16"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="14"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A29" s="16"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="14"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A30" s="16"/>
-      <c r="B30" s="16"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="14"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A31" s="16"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="14"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A32" s="16"/>
-      <c r="B32" s="16"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="14"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A33" s="16"/>
-      <c r="B33" s="16"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="14"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A34" s="16"/>
-      <c r="B34" s="16"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="14"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A35" s="16"/>
-      <c r="B35" s="16"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="14"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A36" s="16"/>
-      <c r="B36" s="16"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="14"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="4"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="4"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A39" s="4"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="4"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A40" s="4"/>
-      <c r="B40" s="4"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="4"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A41" s="4"/>
-      <c r="B41" s="4"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="4"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.15">
-      <c r="A42" s="4"/>
-      <c r="B42" s="4"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>